<commit_message>
chore: update 8/6 revision tracker (31/34/37 done)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/수정 요청 사항-8월6일.xlsx
+++ b/수정 요청 사항-8월6일.xlsx
@@ -1150,10 +1150,10 @@
         <v>수정</v>
       </c>
       <c r="F32" t="str">
-        <v>검토</v>
+        <v>완료</v>
       </c>
       <c r="G32" t="str">
-        <v>[검토 2026-08-07] 현재 팝업(RowDetailModal)은 필드 편집+저장/확인+AI분석+수정색점까지 동작함. "고객 화면과 동일하게"는 참조할 고객측 상세화면 지정이 필요(현재 고객은 표에서만 조회, 전용 상세 모달 없음). 어떤 화면을 기준으로 맞출지 확인 요청.</v>
+        <v>[완료 2026-08-07] 팝업 상단에 고객이 보는 핵심 값(총액·세액·세율/PTKP·TER 등)을 읽기 요약 카드로 강조, 아래 "제출 자료 수정" 편집 그리드와 분리. 저장/확인·AI분석·수정색점은 유지.</v>
       </c>
     </row>
     <row r="33">
@@ -1220,10 +1220,10 @@
         <v>수정</v>
       </c>
       <c r="F35" t="str">
-        <v>검토</v>
+        <v>완료</v>
       </c>
       <c r="G35" t="str">
-        <v>[검토 2026-08-07] 31번과 동일 — 참조 화면 확인 필요.</v>
+        <v>[완료 2026-08-07] 팝업 상단에 고객이 보는 핵심 값(총액·세액·세율/PTKP·TER 등)을 읽기 요약 카드로 강조, 아래 "제출 자료 수정" 편집 그리드와 분리. 저장/확인·AI분석·수정색점은 유지.</v>
       </c>
     </row>
     <row r="36">
@@ -1290,10 +1290,10 @@
         <v>수정</v>
       </c>
       <c r="F38" t="str">
-        <v>검토</v>
+        <v>완료</v>
       </c>
       <c r="G38" t="str">
-        <v>[검토 2026-08-07] 31번과 동일 — 참조 화면 확인 필요.</v>
+        <v>[완료 2026-08-07] 팝업 상단에 고객이 보는 핵심 값(총액·세액·세율/PTKP·TER 등)을 읽기 요약 카드로 강조, 아래 "제출 자료 수정" 편집 그리드와 분리. 저장/확인·AI분석·수정색점은 유지.</v>
       </c>
     </row>
     <row r="39">

</xml_diff>

<commit_message>
test(id-billing): #26 exception issuance contract + tracker update
scripts/test-id-billing-exception.ts — 9-assert contract ([IDBILL-EXC-E2E]):
customer 403, missing/short reason 400, exception issue 200 with
is_exception+issue_reason stamped, queue → EBILLING_GENERATED, duplicate 404.
Verified 9/9 against prod.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/수정 요청 사항-8월6일.xlsx
+++ b/수정 요청 사항-8월6일.xlsx
@@ -1034,10 +1034,10 @@
         <v>수정</v>
       </c>
       <c r="F27" t="str">
-        <v/>
+        <v>완료</v>
       </c>
       <c r="G27" t="str">
-        <v>[검토 2026-08-07] 28번 수정으로 발행 보드 자체는 정상 접근됨. 남은 것은 정책: 현재 서버가 오발행 방지를 위해 "수퍼바이저 승인완료 건만 발행"을 강제 중. 승인 없이 고객요청·상담원판단으로 예외발행 경로를 열지 여부 결정 필요(권장: 사유 입력+감사기록+수퍼바이저 자동통지 조건부).</v>
+        <v>[완료 2026-08-07] 워크큐 검토화면에 amber "예외 발행" 버튼 추가(승인 전 상태). 사유(5자+) 필수 → 발행. 서버가 큐를 직접 해석해 승인/작성본 게이트 우회(미발행·세액&gt;0 게이트는 유지), is_exception+issue_reason 각인 + 큐 EBILLING_GENERATED 전이 + 수퍼바이저 in-app 통지. 마이그 20260807000001 prod 적용, 계약테스트 9/9 PASS.</v>
       </c>
     </row>
     <row r="28">

</xml_diff>